<commit_message>
feat: Implement AI-driven food recommendations based on weather conditions
</commit_message>
<xml_diff>
--- a/microservices/cart_service/data/cart.xlsx
+++ b/microservices/cart_service/data/cart.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,6 +460,111 @@
         <v>90000</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>["b\u00e1nh c\u00e1 ch\u00e0 b\u00f4ng"]</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>[1]</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>["b\u00e1nh c\u00e1 matcha"]</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>["b\u00e1nh c\u00e1 ch\u00e0 b\u00f4ng"]</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>[2]</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>["tr\u00e0 \u0111\u00e0o(size l)"]</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>[1]</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>["b\u00e1nh c\u00e1 ph\u00f4 mai"]</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>[2]</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>["tr\u00e0 chanh(size m)"]</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>[1]</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>["b\u00e1nh b\u00e8o", "b\u00e1nh b\u00e8o", "b\u00e1nh b\u00e8o", "b\u00e1nh b\u00e8o"]</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>[2, 2, 2, 2]</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1200000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>